<commit_message>
Modified SSF bulk file'
</commit_message>
<xml_diff>
--- a/templates/SSF_Entry.xlsx
+++ b/templates/SSF_Entry.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>ปี 2569</t>
   </si>
@@ -38,6 +38,9 @@
   </si>
   <si>
     <t>เลขบัตรประชาชน</t>
+  </si>
+  <si>
+    <t>ประเภท</t>
   </si>
   <si>
     <t>โรงพยาบาล 1</t>
@@ -382,8 +385,8 @@
   <cols>
     <col customWidth="1" min="1" max="5" width="12.63"/>
     <col customWidth="1" min="6" max="6" width="25.13"/>
-    <col customWidth="1" min="7" max="8" width="12.63"/>
-    <col customWidth="1" min="10" max="11" width="25.13"/>
+    <col customWidth="1" min="7" max="9" width="12.63"/>
+    <col customWidth="1" min="11" max="12" width="25.13"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -420,7 +423,7 @@
       <c r="F4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" s="3" t="s">
         <v>9</v>
       </c>
       <c r="H4" s="2" t="s">
@@ -441,7 +444,9 @@
       <c r="M4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="N4" s="4"/>
+      <c r="N4" s="2" t="s">
+        <v>16</v>
+      </c>
       <c r="O4" s="4"/>
       <c r="P4" s="4"/>
       <c r="Q4" s="4"/>
@@ -457,10 +462,11 @@
       <c r="AA4" s="4"/>
       <c r="AB4" s="4"/>
       <c r="AC4" s="4"/>
+      <c r="AD4" s="4"/>
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
@@ -470,14 +476,15 @@
       <c r="G5" s="5"/>
       <c r="H5" s="5"/>
       <c r="I5" s="5"/>
-      <c r="J5" s="7"/>
-      <c r="K5" s="8"/>
-      <c r="L5" s="6"/>
+      <c r="J5" s="5"/>
+      <c r="K5" s="7"/>
+      <c r="L5" s="8"/>
       <c r="M5" s="6"/>
+      <c r="N5" s="6"/>
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
@@ -487,14 +494,15 @@
       <c r="G6" s="5"/>
       <c r="H6" s="5"/>
       <c r="I6" s="5"/>
-      <c r="J6" s="9"/>
+      <c r="J6" s="5"/>
       <c r="K6" s="9"/>
-      <c r="L6" s="6"/>
+      <c r="L6" s="9"/>
       <c r="M6" s="6"/>
+      <c r="N6" s="6"/>
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="5"/>
@@ -504,14 +512,15 @@
       <c r="G7" s="5"/>
       <c r="H7" s="5"/>
       <c r="I7" s="5"/>
-      <c r="J7" s="7"/>
+      <c r="J7" s="5"/>
       <c r="K7" s="7"/>
-      <c r="L7" s="5"/>
+      <c r="L7" s="7"/>
       <c r="M7" s="5"/>
+      <c r="N7" s="5"/>
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="5"/>
@@ -521,14 +530,15 @@
       <c r="G8" s="5"/>
       <c r="H8" s="5"/>
       <c r="I8" s="5"/>
-      <c r="J8" s="7"/>
+      <c r="J8" s="5"/>
       <c r="K8" s="7"/>
-      <c r="L8" s="5"/>
+      <c r="L8" s="7"/>
       <c r="M8" s="5"/>
+      <c r="N8" s="5"/>
     </row>
     <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="5"/>
@@ -538,14 +548,15 @@
       <c r="G9" s="5"/>
       <c r="H9" s="5"/>
       <c r="I9" s="5"/>
-      <c r="J9" s="7"/>
+      <c r="J9" s="5"/>
       <c r="K9" s="7"/>
-      <c r="L9" s="5"/>
+      <c r="L9" s="7"/>
       <c r="M9" s="5"/>
+      <c r="N9" s="5"/>
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="5"/>
@@ -555,14 +566,15 @@
       <c r="G10" s="5"/>
       <c r="H10" s="5"/>
       <c r="I10" s="5"/>
-      <c r="J10" s="7"/>
+      <c r="J10" s="5"/>
       <c r="K10" s="7"/>
-      <c r="L10" s="5"/>
+      <c r="L10" s="7"/>
       <c r="M10" s="5"/>
+      <c r="N10" s="5"/>
     </row>
     <row r="11" ht="15.75" customHeight="1">
       <c r="A11" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B11" s="6"/>
       <c r="C11" s="5"/>
@@ -572,14 +584,15 @@
       <c r="G11" s="5"/>
       <c r="H11" s="5"/>
       <c r="I11" s="5"/>
-      <c r="J11" s="7"/>
+      <c r="J11" s="5"/>
       <c r="K11" s="7"/>
-      <c r="L11" s="5"/>
+      <c r="L11" s="7"/>
       <c r="M11" s="5"/>
+      <c r="N11" s="5"/>
     </row>
     <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="5"/>
@@ -589,14 +602,15 @@
       <c r="G12" s="5"/>
       <c r="H12" s="5"/>
       <c r="I12" s="5"/>
-      <c r="J12" s="7"/>
+      <c r="J12" s="5"/>
       <c r="K12" s="7"/>
-      <c r="L12" s="5"/>
+      <c r="L12" s="7"/>
       <c r="M12" s="5"/>
+      <c r="N12" s="5"/>
     </row>
     <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B13" s="6"/>
       <c r="C13" s="5"/>
@@ -606,14 +620,15 @@
       <c r="G13" s="5"/>
       <c r="H13" s="5"/>
       <c r="I13" s="5"/>
-      <c r="J13" s="7"/>
+      <c r="J13" s="5"/>
       <c r="K13" s="7"/>
-      <c r="L13" s="5"/>
+      <c r="L13" s="7"/>
       <c r="M13" s="5"/>
+      <c r="N13" s="5"/>
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="5"/>
@@ -623,10 +638,11 @@
       <c r="G14" s="5"/>
       <c r="H14" s="5"/>
       <c r="I14" s="5"/>
-      <c r="J14" s="7"/>
+      <c r="J14" s="5"/>
       <c r="K14" s="7"/>
-      <c r="L14" s="5"/>
+      <c r="L14" s="7"/>
       <c r="M14" s="5"/>
+      <c r="N14" s="5"/>
     </row>
     <row r="15" ht="15.75" customHeight="1"/>
     <row r="16" ht="15.75" customHeight="1"/>
@@ -1616,15 +1632,18 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A3:M3"/>
+    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A3:N3"/>
   </mergeCells>
   <dataValidations>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G5:G14">
+      <formula1>"1-03,1-03/1"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B5:B14">
       <formula1>"นาย,นาง,นางสาว"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E5:E14 L5:M14">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E5:E14 M5:N14">
       <formula1>"Imported,Pending,Registered"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>